<commit_message>
Backlog: C1-T5 cross-browser capture confirmed by project lead; Epic C complete
Edge, Firefox and Safari runs confirmed complete by the project lead on
23 Sep; per-run results were not captured, so the probe README records
them as confirmed without recorderMime/verdict detail. Chromium PASS is
the automated run.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RD5kD4obV2Jan7tMKpiqPQ
</commit_message>
<xml_diff>
--- a/Documentation/jira-backlog.xlsx
+++ b/Documentation/jira-backlog.xlsx
@@ -4401,14 +4401,14 @@
           <t>epic</t>
         </is>
       </c>
-      <c r="N57" s="51" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="N57" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="O57" s="36" t="inlineStr">
         <is>
-          <t>12/13 sub-tasks done, 3/4 stories done</t>
+          <t>13/13 sub-tasks done, 4/4 stories done</t>
         </is>
       </c>
       <c r="P57" s="36" t="inlineStr">
@@ -4472,19 +4472,19 @@
           <t>p0,m1</t>
         </is>
       </c>
-      <c r="N58" s="51" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="N58" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="O58" s="36" t="inlineStr">
         <is>
-          <t>4/5 sub-tasks done</t>
+          <t>5/5 sub-tasks done</t>
         </is>
       </c>
       <c r="P58" s="36" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -4787,14 +4787,14 @@
           <t>qa</t>
         </is>
       </c>
-      <c r="N63" s="51" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="N63" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="O63" s="36" t="inlineStr">
         <is>
-          <t>Safari MP4 labelling bug fixed; per-browser format selection + matrix spec; real Chromium capture PASS via web/e2e/capture-probe; Edge, Firefox, Safari manual runs pending (checklist in README)</t>
+          <t>Safari MP4 labelling fixed; per-browser format + matrix spec; Chromium capture PASS (automated, web/e2e/capture-probe); Edge/Firefox/Safari confirmed complete by project lead 2026-09-23 (results not recorded in the probe README)</t>
         </is>
       </c>
       <c r="P63" s="36" t="inlineStr">
@@ -5239,7 +5239,7 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="O70" t="inlineStr">
+      <c r="O70" s="36" t="inlineStr">
         <is>
           <t>resumable-upload.spec (network drop → reload → only missing parts sent; server-authoritative parts; file mismatch; offline wait) + ResumableUploadTest (API)</t>
         </is>
@@ -18432,10 +18432,10 @@
         <v>13</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E6" s="36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" s="36" t="n">
         <v>0</v>
@@ -18444,11 +18444,11 @@
         <v>0</v>
       </c>
       <c r="H6" s="54" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="I6" s="36" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>4/4</t>
         </is>
       </c>
     </row>
@@ -18813,10 +18813,10 @@
         <v>194</v>
       </c>
       <c r="D17" s="39" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E17" s="39" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F17" s="39" t="n">
         <v>12</v>
@@ -18825,7 +18825,7 @@
         <v>6</v>
       </c>
       <c r="H17" s="55" t="n">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="I17" s="39" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Epic I complete: translation links read both ways; stale translations visible in the document list
- I2-T3 (FR-803): Document::source() and translations(); GET /documents/{id}
  and /published return `source` and `translations` ({id, language, title,
  state, translation_stale}), each only when the caller can open it, and the
  published payload lists only translations that are published themselves.
  Reader shows "Translated from XX" / "Also in DE FR*"; editor links to the
  source and its translations; the assist panel refuses a second translation
  in the same language before the server's 409.
- I3-T2 (FR-804): the space browser tags translations with their language
  and "out of date" when the source was re-approved; reader and editor
  banners link to the source.
- Doc 05 v1.5; backlog Epic I 10/10.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RD5kD4obV2Jan7tMKpiqPQ
</commit_message>
<xml_diff>
--- a/Documentation/jira-backlog.xlsx
+++ b/Documentation/jira-backlog.xlsx
@@ -13023,19 +13023,19 @@
           <t>epic</t>
         </is>
       </c>
-      <c r="N191" s="51" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="N191" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="O191" s="36" t="inlineStr">
         <is>
-          <t>8/10 sub-tasks done, 2/4 stories done</t>
+          <t>10/10 sub-tasks done, 4/4 stories done</t>
         </is>
       </c>
       <c r="P191" s="36" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -13106,7 +13106,7 @@
       </c>
       <c r="P192" s="36" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -13357,19 +13357,19 @@
           <t>p1,m4</t>
         </is>
       </c>
-      <c r="N196" s="51" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="N196" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="O196" s="36" t="inlineStr">
         <is>
-          <t>2/3 sub-tasks done</t>
+          <t>3/3 sub-tasks done</t>
         </is>
       </c>
       <c r="P196" s="36" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -13544,19 +13544,19 @@
           <t>database</t>
         </is>
       </c>
-      <c r="N199" s="51" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="N199" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="O199" s="36" t="inlineStr">
         <is>
-          <t>translation_of is one-directional; no back-link list on the source yet</t>
+          <t>Document::source()/translations(); GET /documents/{id} and /published return source + translations (visible, published-only for readers); reader/editor links; assist panel blocks duplicate languages</t>
         </is>
       </c>
       <c r="P199" s="36" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -13611,19 +13611,19 @@
           <t>p2,m4</t>
         </is>
       </c>
-      <c r="N200" s="51" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="N200" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="O200" s="36" t="inlineStr">
         <is>
-          <t>1/2 sub-tasks done</t>
+          <t>2/2 sub-tasks done</t>
         </is>
       </c>
       <c r="P200" s="36" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -13739,19 +13739,19 @@
           <t>frontend</t>
         </is>
       </c>
-      <c r="N202" s="51" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="N202" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="O202" s="36" t="inlineStr">
         <is>
-          <t>reader + editor banner; document list indicator not added</t>
+          <t>reader banner + source link, editor banner + source link, space browser shows language tag and "out of date"</t>
         </is>
       </c>
       <c r="P202" s="36" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -13822,7 +13822,7 @@
       </c>
       <c r="P203" s="36" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -18647,10 +18647,10 @@
         <v>10</v>
       </c>
       <c r="D12" s="36" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E12" s="36" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F12" s="36" t="n">
         <v>0</v>
@@ -18659,11 +18659,11 @@
         <v>0</v>
       </c>
       <c r="H12" s="54" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="I12" s="36" t="inlineStr">
         <is>
-          <t>2/4</t>
+          <t>4/4</t>
         </is>
       </c>
     </row>
@@ -18818,10 +18818,10 @@
         <v>194</v>
       </c>
       <c r="D17" s="39" t="n">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="E17" s="39" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F17" s="39" t="n">
         <v>7</v>
@@ -18830,7 +18830,7 @@
         <v>11</v>
       </c>
       <c r="H17" s="55" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="I17" s="39" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Backlog: status review 2026-09-24 — 183/194 done, 11 blocked; "what unblocks it" sheet
CI on GitHub is green for 2dbd6f7 (all three jobs). The Deploy workflow
failed only at doctl authentication because the DigitalOcean token and
app ids are not set yet (M3-T2). New sheet lists each blocked item with
what is already built, what unblocks it, who, and the command to run.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RD5kD4obV2Jan7tMKpiqPQ
</commit_message>
<xml_diff>
--- a/Documentation/jira-backlog.xlsx
+++ b/Documentation/jira-backlog.xlsx
@@ -9,10 +9,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jira Import" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epic Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestone Plan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Component Load" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Guide" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocked — what unblocks it" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epic Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestone Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Component Load" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Guide" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Jira Import'!$A$1:$M$273</definedName>
@@ -27,7 +28,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -99,6 +100,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="9">
@@ -181,7 +186,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -405,6 +410,10 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -5559,12 +5568,12 @@
       </c>
       <c r="O75" s="36" t="inlineStr">
         <is>
-          <t>17/22 sub-tasks done, 3/6 stories done; the rest need real recordings / provider keys</t>
+          <t>17/22 sub-tasks done, 3/6 stories done; remaining sub-tasks are Blocked (see 'Blocked — what unblocks it')</t>
         </is>
       </c>
       <c r="P75" s="36" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -9865,12 +9874,12 @@
       </c>
       <c r="O142" s="36" t="inlineStr">
         <is>
-          <t>16/19 sub-tasks done, 3/6 stories done; the rest need the DO droplet and design-partner content</t>
+          <t>16/19 sub-tasks done, 3/6 stories done; remaining sub-tasks are Blocked (see 'Blocked — what unblocks it')</t>
         </is>
       </c>
       <c r="P142" s="36" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -11548,12 +11557,12 @@
       </c>
       <c r="O168" s="36" t="inlineStr">
         <is>
-          <t>15/16 sub-tasks done, 5/6 stories done; refusal eval needs API keys on staging</t>
+          <t>15/16 sub-tasks done, 5/6 stories done; remaining sub-tasks are Blocked (see 'Blocked — what unblocks it')</t>
         </is>
       </c>
       <c r="P168" s="36" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -15013,12 +15022,12 @@
       </c>
       <c r="O222" s="36" t="inlineStr">
         <is>
-          <t>10/11 sub-tasks done, 3/4 stories done; only the payment-provider driver remains, blocked on the provider decision</t>
+          <t>10/11 sub-tasks done, 3/4 stories done; remaining sub-tasks are Blocked (see 'Blocked — what unblocks it')</t>
         </is>
       </c>
       <c r="P222" s="36" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -16881,12 +16890,12 @@
       </c>
       <c r="O251" s="36" t="inlineStr">
         <is>
-          <t>16/17 sub-tasks done, 4/5 stories done; only provisioning in the DO account remains</t>
+          <t>16/17 sub-tasks done, 4/5 stories done; remaining sub-tasks are Blocked (see 'Blocked — what unblocks it')</t>
         </is>
       </c>
       <c r="P251" s="36" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -17785,7 +17794,7 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="O265" t="inlineStr">
+      <c r="O265" s="36" t="inlineStr">
         <is>
           <t>sentry/sentry-laravel (Integration::handles) + @sentry/angular loaded lazily behind a build-time DSN; release = commit via CD, environment tag; TrackingErrorHandler queues early errors</t>
         </is>
@@ -17913,7 +17922,7 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="O267" t="inlineStr">
+      <c r="O267" s="36" t="inlineStr">
         <is>
           <t>Ops\Metrics + GET /internal/metrics (bearer METRICS_TOKEN, Prometheus text): stage success/p50/p95, cost per SOP, index backlog, chat refusal/latency; infra/monitoring Grafana dashboard + rules</t>
         </is>
@@ -17977,7 +17986,7 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="O268" t="inlineStr">
+      <c r="O268" s="36" t="inlineStr">
         <is>
           <t>ops:check-health every 10 min: generation failure rate &gt; 25% (halts excluded), embedding backlog (&gt;10 docs, &gt;60 min, failed index jobs) → alerts channel, once an hour; unindexed docs via retrieval:check-index</t>
         </is>
@@ -18331,7 +18340,7 @@
     <row r="1">
       <c r="A1" s="39" t="inlineStr">
         <is>
-          <t>Progress as of 2026-09-23 — derived from the Status column on 'Jira Import'</t>
+          <t>Progress as of 2026-09-24 — derived from the Status column on 'Jira Import'. CI on GitHub is green for commit 2dbd6f7 (all three jobs: API on SQLite, API on MySQL 8.4 incl. tenancy suite, rollback drill and real Qdrant, and web lint/test/build).</t>
         </is>
       </c>
     </row>
@@ -18880,7 +18889,7 @@
       </c>
       <c r="B20" s="36" t="inlineStr">
         <is>
-          <t>built, lint-clean, unit/feature tests written. As of 2026-09-23 the API passes the raw-query check, Pint, PHPStan level 6 and all 115 PHPUnit tests on SQLite and on MySQL 8.4 locally; the web app passes lint, 40 tests and the production build; CI confirmation pending the push</t>
+          <t>built, lint-clean, tests written and passing; confirmed by CI on GitHub for 2dbd6f7 (API 115 tests on SQLite and MySQL 8.4, PHPStan level 6, Pint, raw-query check, Qdrant integration, migration rollback drill; web lint, 40 tests, production build)</t>
         </is>
       </c>
     </row>
@@ -18916,7 +18925,7 @@
       </c>
       <c r="B23" s="36" t="inlineStr">
         <is>
-          <t>waiting on a decision, keys or material from the team (transcription provider, billing provider, real recordings)</t>
+          <t>cannot be finished by development alone — needs a decision, an account, keys or real content from the team; see the 'Blocked — what unblocks it' sheet</t>
         </is>
       </c>
     </row>
@@ -18934,6 +18943,480 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" style="37" min="1" max="1"/>
+    <col width="6" customWidth="1" style="37" min="2" max="2"/>
+    <col width="34" customWidth="1" style="37" min="3" max="3"/>
+    <col width="52" customWidth="1" style="37" min="4" max="4"/>
+    <col width="60" customWidth="1" style="37" min="5" max="5"/>
+    <col width="22" customWidth="1" style="37" min="6" max="6"/>
+    <col width="52" customWidth="1" style="37" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="80" t="inlineStr">
+        <is>
+          <t>Blocked items as of 2026-09-24 — everything development could build is done; each row needs one thing from the team</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="39" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="B3" s="39" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="C3" s="39" t="inlineStr">
+        <is>
+          <t>Sub-task</t>
+        </is>
+      </c>
+      <c r="D3" s="39" t="inlineStr">
+        <is>
+          <t>What is already built</t>
+        </is>
+      </c>
+      <c r="E3" s="39" t="inlineStr">
+        <is>
+          <t>What unblocks it</t>
+        </is>
+      </c>
+      <c r="F3" s="39" t="inlineStr">
+        <is>
+          <t>Who</t>
+        </is>
+      </c>
+      <c r="G3" s="39" t="inlineStr">
+        <is>
+          <t>Then run</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="81" t="inlineStr">
+        <is>
+          <t>D0-T1</t>
+        </is>
+      </c>
+      <c r="B4" s="81" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C4" s="81" t="inlineStr">
+        <is>
+          <t>Assemble 10-recording evaluation set</t>
+        </is>
+      </c>
+      <c r="D4" s="81" t="inlineStr">
+        <is>
+          <t>eval-set.csv lists the 20 slots to cover; pipeline:eval runs them</t>
+        </is>
+      </c>
+      <c r="E4" s="81" t="inlineStr">
+        <is>
+          <t>10 real screen recordings, narrated, unscripted (spike/generation-eval/eval-set.csv slots 1–10)</t>
+        </is>
+      </c>
+      <c r="F4" s="81" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="G4" s="81" t="inlineStr">
+        <is>
+          <t>php artisan pipeline:eval &lt;folder&gt; --mock  (harness check), then with keys</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="81" t="inlineStr">
+        <is>
+          <t>D0-T2</t>
+        </is>
+      </c>
+      <c r="B5" s="81" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C5" s="81" t="inlineStr">
+        <is>
+          <t>Benchmark Whisper API vs Deepgram</t>
+        </is>
+      </c>
+      <c r="D5" s="81" t="inlineStr">
+        <is>
+          <t>Both drivers, side-by-side run, cost and timestamp columns in runs.csv</t>
+        </is>
+      </c>
+      <c r="E5" s="81" t="inlineStr">
+        <is>
+          <t>OPENAI_API_KEY and DEEPGRAM_API_KEY on staging + the recordings above</t>
+        </is>
+      </c>
+      <c r="F5" s="81" t="inlineStr">
+        <is>
+          <t>Project lead</t>
+        </is>
+      </c>
+      <c r="G5" s="81" t="inlineStr">
+        <is>
+          <t>php artisan pipeline:eval &lt;folder&gt; --providers=whisper,deepgram; python score.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="81" t="inlineStr">
+        <is>
+          <t>D0-T3</t>
+        </is>
+      </c>
+      <c r="B6" s="81" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C6" s="81" t="inlineStr">
+        <is>
+          <t>Confirm zero-retention terms</t>
+        </is>
+      </c>
+      <c r="D6" s="81" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="81" t="inlineStr">
+        <is>
+          <t>Choose the provider from the benchmark, then written confirmation from the vendor (BRD D5)</t>
+        </is>
+      </c>
+      <c r="F6" s="81" t="inlineStr">
+        <is>
+          <t>Project lead</t>
+        </is>
+      </c>
+      <c r="G6" s="81" t="inlineStr">
+        <is>
+          <t>set TRANSCRIPTION_DRIVER=whisper|deepgram in App Platform</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="81" t="inlineStr">
+        <is>
+          <t>D2-T4</t>
+        </is>
+      </c>
+      <c r="B7" s="81" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C7" s="81" t="inlineStr">
+        <is>
+          <t>Segmentation accuracy eval</t>
+        </is>
+      </c>
+      <c r="D7" s="81" t="inlineStr">
+        <is>
+          <t>segments-review.csv written per run; score.py reports boundary precision/recall/F1 ±2 s</t>
+        </is>
+      </c>
+      <c r="E7" s="81" t="inlineStr">
+        <is>
+          <t>The 20 recordings + a reviewer marking human boundaries</t>
+        </is>
+      </c>
+      <c r="F7" s="81" t="inlineStr">
+        <is>
+          <t>Team + reviewer</t>
+        </is>
+      </c>
+      <c r="G7" s="81" t="inlineStr">
+        <is>
+          <t>python spike/generation-eval/score.py --out &lt;out&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="81" t="inlineStr">
+        <is>
+          <t>D4-T5</t>
+        </is>
+      </c>
+      <c r="B8" s="81" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C8" s="81" t="inlineStr">
+        <is>
+          <t>Generation eval set (20 recordings)</t>
+        </is>
+      </c>
+      <c r="D8" s="81" t="inlineStr">
+        <is>
+          <t>pipeline:eval writes draft.md, frames, metrics; human-review.csv per run</t>
+        </is>
+      </c>
+      <c r="E8" s="81" t="inlineStr">
+        <is>
+          <t>The 20 recordings + a reviewer filling human-review.csv (verdict, step count, frames ok)</t>
+        </is>
+      </c>
+      <c r="F8" s="81" t="inlineStr">
+        <is>
+          <t>Team + reviewer</t>
+        </is>
+      </c>
+      <c r="G8" s="81" t="inlineStr">
+        <is>
+          <t>python spike/generation-eval/score.py --out &lt;out&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="81" t="inlineStr">
+        <is>
+          <t>G0-T2</t>
+        </is>
+      </c>
+      <c r="B9" s="81" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="C9" s="81" t="inlineStr">
+        <is>
+          <t>Stand up Qdrant on DigitalOcean</t>
+        </is>
+      </c>
+      <c r="D9" s="81" t="inlineStr">
+        <is>
+          <t>infra/qdrant: compose (v1.19.1 + Caddy TLS), cloud-init, nightly snapshots, runbook; QdrantStore proven against real Qdrant in CI</t>
+        </is>
+      </c>
+      <c r="E9" s="81" t="inlineStr">
+        <is>
+          <t>Create droplet, volume, DNS and firewall in the DO account (infra/qdrant/README.md steps 1–5); set QDRANT_URL / QDRANT_API_KEY / OPENAI_API_KEY in App Platform</t>
+        </is>
+      </c>
+      <c r="F9" s="81" t="inlineStr">
+        <is>
+          <t>Ops (DO account owner)</t>
+        </is>
+      </c>
+      <c r="G9" s="81" t="inlineStr">
+        <is>
+          <t>php artisan vector:ensure-collection; php artisan retrieval:check-index --dry-run</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="81" t="inlineStr">
+        <is>
+          <t>G2-T3</t>
+        </is>
+      </c>
+      <c r="B10" s="81" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="C10" s="81" t="inlineStr">
+        <is>
+          <t>Relevance eval set (50 + 15 questions)</t>
+        </is>
+      </c>
+      <c r="D10" s="81" t="inlineStr">
+        <is>
+          <t>retrieval:eval harness, demo corpus + demo set, retrieval:seed-corpus, doc 08 targets in summary.md</t>
+        </is>
+      </c>
+      <c r="E10" s="81" t="inlineStr">
+        <is>
+          <t>Design-partner content and 50 answerable + 15 unanswerable questions in spike/retrieval-eval format</t>
+        </is>
+      </c>
+      <c r="F10" s="81" t="inlineStr">
+        <is>
+          <t>Project lead + design partner</t>
+        </is>
+      </c>
+      <c r="G10" s="81" t="inlineStr">
+        <is>
+          <t>php artisan retrieval:eval set.json --workspace=&lt;slug&gt; --as=&lt;email&gt; --answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="81" t="inlineStr">
+        <is>
+          <t>G3-T3</t>
+        </is>
+      </c>
+      <c r="B11" s="81" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="C11" s="81" t="inlineStr">
+        <is>
+          <t>Ranking quality eval</t>
+        </is>
+      </c>
+      <c r="D11" s="81" t="inlineStr">
+        <is>
+          <t>retrieval:eval compares fusion weights side by side (--weights)</t>
+        </is>
+      </c>
+      <c r="E11" s="81" t="inlineStr">
+        <is>
+          <t>The eval set from G2-T3</t>
+        </is>
+      </c>
+      <c r="F11" s="81" t="inlineStr">
+        <is>
+          <t>Project lead</t>
+        </is>
+      </c>
+      <c r="G11" s="81" t="inlineStr">
+        <is>
+          <t>php artisan retrieval:eval ... --weights=1:0.6,1:0.3,1:1,1:0,0:1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="81" t="inlineStr">
+        <is>
+          <t>H3-T3</t>
+        </is>
+      </c>
+      <c r="B12" s="81" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="C12" s="81" t="inlineStr">
+        <is>
+          <t>Refusal eval (15 unanswerable questions)</t>
+        </is>
+      </c>
+      <c r="D12" s="81" t="inlineStr">
+        <is>
+          <t>demo/set.json has 15 unanswerable; --answer checks assistant refusal + citations</t>
+        </is>
+      </c>
+      <c r="E12" s="81" t="inlineStr">
+        <is>
+          <t>OPENAI_API_KEY + ANTHROPIC_API_KEY on staging, demo corpus seeded</t>
+        </is>
+      </c>
+      <c r="F12" s="81" t="inlineStr">
+        <is>
+          <t>Project lead</t>
+        </is>
+      </c>
+      <c r="G12" s="81" t="inlineStr">
+        <is>
+          <t>retrieval:seed-corpus demo/corpus.json ...; retrieval:eval demo/set.json ... --answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="81" t="inlineStr">
+        <is>
+          <t>K2-T1</t>
+        </is>
+      </c>
+      <c r="B13" s="81" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="C13" s="81" t="inlineStr">
+        <is>
+          <t>Payment provider integration and webhooks</t>
+        </is>
+      </c>
+      <c r="D13" s="81" t="inlineStr">
+        <is>
+          <t>BillingProvider interface, subscriptions table, plan-change rules, scheduled downgrades, webhook endpoint, Null + Fake drivers, S22 plan chooser</t>
+        </is>
+      </c>
+      <c r="E13" s="81" t="inlineStr">
+        <is>
+          <t>Decide the provider (Stripe / Paddle / …) — open decision 03 §12; then one driver class implementing BillingProvider</t>
+        </is>
+      </c>
+      <c r="F13" s="81" t="inlineStr">
+        <is>
+          <t>CEO / project lead</t>
+        </is>
+      </c>
+      <c r="G13" s="81" t="inlineStr">
+        <is>
+          <t>set BILLING_DRIVER=&lt;provider&gt;, BILLING_WEBHOOK_SECRET; run PlanChangeTest against the real driver</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="81" t="inlineStr">
+        <is>
+          <t>M3-T2</t>
+        </is>
+      </c>
+      <c r="B14" s="81" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C14" s="81" t="inlineStr">
+        <is>
+          <t>Managed MySQL and Valkey with TLS</t>
+        </is>
+      </c>
+      <c r="D14" s="81" t="inlineStr">
+        <is>
+          <t>app.yaml + app.production.yaml, provisioning runbook, CD workflow, rollback drill</t>
+        </is>
+      </c>
+      <c r="E14" s="81" t="inlineStr">
+        <is>
+          <t>Run infra/runbooks/provisioning.md in the DO account; add GitHub secrets DIGITALOCEAN_ACCESS_TOKEN, DO_STAGING_APP_ID, DO_PRODUCTION_APP_ID and the "production" environment with reviewers</t>
+        </is>
+      </c>
+      <c r="F14" s="81" t="inlineStr">
+        <is>
+          <t>Ops (DO account owner)</t>
+        </is>
+      </c>
+      <c r="G14" s="81" t="inlineStr">
+        <is>
+          <t>re-run the Deploy workflow (it failed at doctl auth on 23 Sep because the token is not set yet)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19540,7 +20023,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19822,7 +20305,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20037,7 +20520,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>